<commit_message>
Fix Details links: embed assignment detail sheets inside the workbook
Excel cannot open external URLs or local .md paths from a standalone downloaded
.xlsx (shows 'Cannot open the specified file'). Each assignment now gets its
own detail sheet tab inside the same file, with internal HYPERLINK formulas and
a back link to the class summary sheet. Regenerate output/.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/skills/syllabus-dissector/example_output/syllabi.xlsx
+++ b/.cursor/skills/syllabus-dissector/example_output/syllabi.xlsx
@@ -8,7 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATH-201" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Sleep Paper" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Witchcraft Paper" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Mid-term" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Final Exam" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Discussion Section" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Identification Quizzes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103-Extra Credit" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATH-201" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATH-201-Homework" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATH-201-Final Project" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATH-201-Midterm" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +55,25 @@
     <font>
       <color rgb="000563C1"/>
       <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00D62728"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002CA02C"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="8">
@@ -111,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -139,6 +168,20 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -163,6 +206,7 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -653,10 +697,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F8" s="7">
+        <f>HYPERLINK("#'HIST-103-Sleep Paper'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -685,10 +728,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F9" s="10">
+        <f>HYPERLINK("#'HIST-103-Witchcraft Paper'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -717,10 +759,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F10" s="7">
+        <f>HYPERLINK("#'HIST-103-Mid-term'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -749,10 +790,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F11" s="10">
+        <f>HYPERLINK("#'HIST-103-Final Exam'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -781,10 +821,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F12" s="7">
+        <f>HYPERLINK("#'HIST-103-Discussion Section'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -813,10 +852,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F13" s="10">
+        <f>HYPERLINK("#'HIST-103-Identification Quizzes'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -845,10 +883,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F14" s="7">
+        <f>HYPERLINK("#'HIST-103-Extra Credit'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -868,20 +905,909 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId7"/>
-  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00A0D4A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'MATH-201'!A1","← Back to MATH-201")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** MATH-201</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 450 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-12-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Weekly problem sets.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00A0D4A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'MATH-201'!A1","← Back to MATH-201")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Final Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Final Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** MATH-201</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 300 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-12-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Group project, teams of 3.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00A0D4A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'MATH-201'!A1","← Back to MATH-201")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Midterm</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Midterm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** MATH-201</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 250 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Covers chapters 1-5.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Sleep Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Sleep Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>- **Notes:** Turned in via TA's Brightspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>4-page paper using Ekirch 'Sleep we have lost' and Handley chapters. Pick ONE prompt about sleep and power/primary sources. Due 11:59pm via TA's Brightspace. Requires thesis, topic sentences, and at least two quotes/references per paragraph with citations.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Witchcraft Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Witchcraft Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-11-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-11-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>4-page paper using Brian Levack's The Witchcraft Sourcebook. Pick ONE prompt about witchcraft accusations, gender, or power. Due Nov 10 at 11:59pm via TA's Brightspace. Do not search the internet; cite only Levack or lecture.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Mid-term</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Mid-term</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>In-class exam. Part 1 (30%): ten identifications. Part 2 (70%): one essay chosen from two of five pre-released prompts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-12-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>In-class exam, same format as midterm: 10 identifications (30%) and one longer essay (70%) from pre-released prompts. Dec 10, 4:30-6:30pm, THH 301.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Discussion Section</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Discussion Section</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-12-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>- **Notes:** Ongoing participation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Participation grade set by TA. Includes two primary source activities (Nov 13 and Nov 20) turned into TA's Brightspace, graded pass/fail.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Identification Quizzes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Identification Quizzes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-12-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>- **Notes:** Lowest score dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Eleven quizzes at the start of class asking you to identify two of three listed terms. Cannot be made up; lowest score dropped.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00EC9D9E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11">
+        <f>HYPERLINK("#'HIST-103'!A1","← Back to HIST-103")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Extra Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Extra Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>- **Class:** HIST-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>- **Weight:** —</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>- **Start date:** 2025-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>- **Due date:** 2025-12-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>- **Group project:** No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>- **Notes:** Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Up to two 'Experiencing the Past' activities. Each gives two extra points on a paper. Email to TA by Dec 4.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002CA02C"/>
@@ -900,7 +1826,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>MATH-201 — Linear Algebra</t>
         </is>
@@ -955,131 +1881,128 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Group Project</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>450 pts</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>2025-12-01</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F8" s="21">
+        <f>HYPERLINK("#'MATH-201-Homework'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Final Project</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>300 pts</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>2025-12-05</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F9" s="24">
+        <f>HYPERLINK("#'MATH-201-Final Project'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Midterm</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>2025-10-15</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>Open details</t>
-        </is>
+      <c r="F10" s="21">
+        <f>HYPERLINK("#'MATH-201-Midterm'!A1","Open details")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1099,11 +2022,6 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use hosted PDF URLs in HYPERLINK formulas — no zip required
Excel cannot open relative local PDF paths from a standalone downloaded xlsx.
Point Open PDF cells at raw GitHub-hosted PDF URLs via HYPERLINK formulas so
clicking opens the document in the browser from a single downloaded workbook.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/skills/syllabus-dissector/example_output/syllabi.xlsx
+++ b/.cursor/skills/syllabus-dissector/example_output/syllabi.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -116,6 +116,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -605,30 +617,29 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>2025-09-04</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F8" s="16">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -637,30 +648,29 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>2025-11-06</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>2025-11-10</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F9" s="18">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -669,30 +679,29 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>2025-10-06</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F10" s="16">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -701,30 +710,29 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>2025-10-13</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>2025-12-10</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F11" s="18">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -733,30 +741,29 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F12" s="16">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -765,30 +772,29 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>2025-12-03</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F13" s="18">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -797,30 +803,29 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>Open PDF</t>
-        </is>
+      <c r="F14" s="16">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -840,15 +845,6 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId7"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix PDF layout: organized sections, proper spacing, no text fragments
Rewrite PDF generator with consistent margins, accent section headers, label/value
summary rows, hanging-indent bullets, and set_x resets to fix fpdf2 multi_cell
bugs that caused text fragments on the right margin.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/skills/syllabus-dissector/example_output/syllabi.xlsx
+++ b/.cursor/skills/syllabus-dissector/example_output/syllabi.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -116,6 +116,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -617,27 +641,27 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>2025-09-04</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="24">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -648,27 +672,27 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>2025-11-06</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>2025-11-10</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="26">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -679,27 +703,27 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>2025-10-06</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="24">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -710,27 +734,27 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>2025-10-13</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="25" t="inlineStr">
         <is>
           <t>2025-12-10</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="26">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -741,27 +765,27 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="24">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -772,27 +796,27 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="25" t="inlineStr">
         <is>
           <t>2025-12-03</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="26">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -803,27 +827,27 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>2025-08-25</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>2025-12-04</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="24">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
         <v/>
       </c>

</xml_diff>